<commit_message>
IA builds: nearby reach 6 nodes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XYUkSSUbVnaTPPLQ7pEPnZ
</commit_message>
<xml_diff>
--- a/z6_con/IA_BUILDS_BASE_CASE.xlsx
+++ b/z6_con/IA_BUILDS_BASE_CASE.xlsx
@@ -764,7 +764,7 @@
       </c>
       <c r="V5" s="4" t="inlineStr">
         <is>
-          <t>&lt;=5 nodes</t>
+          <t>&lt;=6 nodes</t>
         </is>
       </c>
       <c r="W5" s="6" t="n">
@@ -884,7 +884,7 @@
       </c>
       <c r="V6" s="4" t="inlineStr">
         <is>
-          <t>&lt;=5 nodes</t>
+          <t>&lt;=6 nodes</t>
         </is>
       </c>
       <c r="W6" s="6" t="n">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="V7" s="4" t="inlineStr">
         <is>
-          <t>&lt;=5 nodes</t>
+          <t>&lt;=6 nodes</t>
         </is>
       </c>
       <c r="W7" s="6" t="n">
@@ -1019,10 +1019,10 @@
       <c r="Z7" s="7" t="n">
         <v>0.1407</v>
       </c>
-      <c r="AA7" s="4" t="n">
+      <c r="AA7" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="AB7" s="5" t="n">
+      <c r="AB7" s="7" t="n">
         <v>0.0641</v>
       </c>
       <c r="AC7" s="4" t="n">
@@ -1124,7 +1124,7 @@
       </c>
       <c r="V8" s="4" t="inlineStr">
         <is>
-          <t>&lt;=5 nodes</t>
+          <t>&lt;=6 nodes</t>
         </is>
       </c>
       <c r="W8" s="4" t="n">
@@ -1244,7 +1244,7 @@
       </c>
       <c r="V9" s="4" t="inlineStr">
         <is>
-          <t>&lt;=5 nodes</t>
+          <t>&lt;=6 nodes</t>
         </is>
       </c>
       <c r="W9" s="4" t="n">
@@ -1273,98 +1273,98 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="n">
+      <c r="A10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>GEN-2023-033</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>DISIS-2023-001</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Clay</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>MO</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>WERE</t>
         </is>
       </c>
-      <c r="G10" s="8" t="n">
+      <c r="G10" s="4" t="n">
         <v>536</v>
       </c>
-      <c r="H10" s="8" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>WERE</t>
         </is>
       </c>
-      <c r="I10" s="8" t="n">
+      <c r="I10" s="4" t="n">
         <v>541248</v>
       </c>
-      <c r="J10" s="8" t="inlineStr">
+      <c r="J10" s="4" t="inlineStr">
         <is>
           <t>LBRTYST5</t>
         </is>
       </c>
-      <c r="K10" s="8" t="n">
+      <c r="K10" s="4" t="n">
         <v>161</v>
       </c>
-      <c r="L10" s="8" t="inlineStr">
+      <c r="L10" s="4" t="inlineStr">
         <is>
           <t>Liberty South 161 kV</t>
         </is>
       </c>
-      <c r="M10" s="8" t="inlineStr">
+      <c r="M10" s="4" t="inlineStr">
         <is>
           <t>Battery/Storage</t>
         </is>
       </c>
-      <c r="N10" s="8" t="inlineStr">
+      <c r="N10" s="4" t="inlineStr">
         <is>
           <t>ER/NR</t>
         </is>
       </c>
-      <c r="O10" s="8" t="n">
+      <c r="O10" s="4" t="n">
         <v>200</v>
       </c>
-      <c r="P10" s="8" t="n">
+      <c r="P10" s="4" t="n">
         <v>200</v>
       </c>
-      <c r="Q10" s="8" t="inlineStr">
+      <c r="Q10" s="4" t="inlineStr">
         <is>
           <t>4/15/2028</t>
         </is>
       </c>
-      <c r="R10" s="8" t="inlineStr">
+      <c r="R10" s="4" t="inlineStr">
         <is>
           <t>1/7/2028</t>
         </is>
       </c>
-      <c r="S10" s="8" t="inlineStr">
+      <c r="S10" s="4" t="inlineStr">
         <is>
           <t>EmpirePrairie</t>
         </is>
       </c>
-      <c r="T10" s="8" t="n">
+      <c r="T10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="U10" s="9" t="n">
+      <c r="U10" s="5" t="n">
         <v>0.1391</v>
       </c>
-      <c r="V10" s="8" t="inlineStr">
-        <is>
-          <t>added (electrically close)</t>
+      <c r="V10" s="4" t="inlineStr">
+        <is>
+          <t>&lt;=6 nodes</t>
         </is>
       </c>
       <c r="W10" s="4" t="n">
@@ -1385,10 +1385,10 @@
       <c r="AB10" s="5" t="n">
         <v>0.3384</v>
       </c>
-      <c r="AC10" s="4" t="n">
+      <c r="AC10" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="AD10" s="5" t="n">
+      <c r="AD10" s="7" t="n">
         <v>0.1391</v>
       </c>
     </row>
@@ -1484,7 +1484,7 @@
       </c>
       <c r="V11" s="8" t="inlineStr">
         <is>
-          <t>added</t>
+          <t>added (7 nodes)</t>
         </is>
       </c>
       <c r="W11" s="4" t="n">
@@ -1512,25 +1512,13 @@
         <v>0.1798</v>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
       <c r="B13" s="10" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
       <c r="O13" s="10">
         <f>SUM(O5:O11)</f>
         <v/>
@@ -1540,16 +1528,15 @@
         <v/>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Green = within 5 nodes of that project. Yellow row = added beyond the 5-node rule.</t>
+          <t>Green = within 6 nodes of that project. Yellow row = added beyond the 6-node rule.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
           <t>Left out: GEN-2023-037 Nearman, GEN-2023-034 Clear Water-Waco, GEN-2023-061 Carthage (&gt;= 7 nodes and &gt;= 0.18 pu from every project).</t>

</xml_diff>